<commit_message>
restore: bring all files from master (zip backup)
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Test_Case_Report_FE.xlsx
+++ b/Docs/QA-Testing/Test_Case_Report_FE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B400B8-F56B-4D4F-ACA3-598265FD1856}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8DA1A4-6727-469F-97A7-339498B88685}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23490" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="220">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -902,6 +902,9 @@
   </si>
   <si>
     <t>SCRUM-45</t>
+  </si>
+  <si>
+    <t>CodeceptJS cũng fail đúng kỳ vọng (bug giá âm vẫn tồn tại)</t>
   </si>
 </sst>
 </file>
@@ -1502,7 +1505,7 @@
     <col min="8" max="8" width="16.28515625" style="1" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="16.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="21.5703125" style="1" customWidth="1"/>
     <col min="12" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
@@ -2508,7 +2511,9 @@
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
-      <c r="K38" s="3"/>
+      <c r="K38" s="5" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="39" spans="1:11" ht="148.5" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">

</xml_diff>

<commit_message>
SCRUM-77: fix cart quantity + logbug các bug còn lại
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Test_Case_Report_FE.xlsx
+++ b/Docs/QA-Testing/Test_Case_Report_FE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20398"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\MouseWithoutBorders\sss\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiemChungPhanMem\Docs\QA-Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645135DC-B133-4DD6-A701-F45241760765}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C33D1E3-AB95-42CB-A3D1-3C7E9A057C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="226">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -299,9 +299,6 @@
 3. Truy cập /cart, xác nhận sản phẩm có trong local cart. 
 4. Nhấn Sign In, đăng nhập customer1@email.com / 123. 
 5. Truy cập /cart.</t>
-  </si>
-  <si>
-    <t>Sản phẩm trong local cart (B0001, sl=1) được merge vào server cart (POST /cart). Trang giỏ hàng hiển thị B0001 với số lượng = 1. Cookie local cart bị xóa. (REQ-CART-02)</t>
   </si>
   <si>
     <t>TC_FE_CUS_CHK_01</t>
@@ -685,9 +682,6 @@
 8. Kiểm tra giá của sản phẩm vừa chỉnh sửa.</t>
   </si>
   <si>
-    <t>SCRUM-44</t>
-  </si>
-  <si>
     <t>TC_FE_MGR_04</t>
   </si>
   <si>
@@ -907,9 +901,6 @@
     <t>Assertion $40.00 thất bại vì subtotal hiển thị $40,140.00 (dữ liệu giỏ / format số bị ảnh hưởng bởi data BVA trước đó hoặc locale). Không phải bug nghiệp vụ Add to Cart. Cần reset DB hoặc sửa expected linh hoạt hơn trước khi retest.</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Sau Checkout hệ thống chuyển về trang chủ (Get Whatever You Want!). Test vẫn expect thấy "Spring In Action" trên trang sau checkout → sai expected. Hành vi thực tế đúng (cart cleared, redirect home). Sửa test: expect trang chủ hoặc thông báo thành công, không expect tên SP trên /cart nữa.</t>
   </si>
   <si>
@@ -920,13 +911,25 @@
   </si>
   <si>
     <t>Xác nhận lại bug giá âm (Employee) – form không chặn. Cùng root cause SCRUM-44 (Manager).</t>
+  </si>
+  <si>
+    <t>Guest không được thêm vào cart. Chỉ Customer đã login mới thêm được. Local cart không còn hỗ trợ.</t>
+  </si>
+  <si>
+    <t>SCRUM-79</t>
+  </si>
+  <si>
+    <t>SCRUM-80</t>
+  </si>
+  <si>
+    <t>SCRUM-44(đã fix)-SCRUM-81(chưa fix)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -957,14 +960,6 @@
       <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="163"/>
     </font>
   </fonts>
   <fills count="17">
@@ -1092,7 +1087,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1218,12 +1213,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1234,12 +1223,12 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFE699"/>
       <color rgb="FFC6E0B4"/>
       <color rgb="FFFCE4D6"/>
       <color rgb="FFF4B084"/>
       <color rgb="FFDDEBF7"/>
       <color rgb="FF9BC2E6"/>
-      <color rgb="FFFFE699"/>
       <color rgb="FFFFD966"/>
       <color rgb="FF000000"/>
     </mruColors>
@@ -1519,23 +1508,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K48"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="16.5" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="16.8" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="7" customWidth="1"/>
+    <col min="1" max="1" width="27.6640625" style="7" customWidth="1"/>
     <col min="2" max="2" width="36" style="6" customWidth="1"/>
-    <col min="3" max="3" width="30.140625" style="6" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="4" max="4" width="52.85546875" style="6" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="47.85546875" style="6" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="6" width="12.140625" style="1" customWidth="1" collapsed="1"/>
-    <col min="7" max="7" width="20.85546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.7109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16.140625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.85546875" style="1"/>
+    <col min="3" max="3" width="30.109375" style="6" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="52.88671875" style="6" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="47.88671875" style="6" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="12.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13.6640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="21.5546875" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
@@ -1552,25 +1541,25 @@
         <v>4</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G1" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="H1" s="27" t="s">
+        <v>208</v>
+      </c>
+      <c r="I1" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="J1" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="I1" s="27" t="s">
+      <c r="K1" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="J1" s="27" t="s">
-        <v>212</v>
-      </c>
-      <c r="K1" s="27" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>5</v>
       </c>
@@ -1585,7 +1574,7 @@
       <c r="J2" s="30"/>
       <c r="K2" s="30"/>
     </row>
-    <row r="3" spans="1:11" ht="99" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -1602,17 +1591,17 @@
         <v>9</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" ht="99" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A4" s="31" t="s">
         <v>10</v>
       </c>
@@ -1629,17 +1618,17 @@
         <v>14</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H4" s="31"/>
       <c r="I4" s="31"/>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
     </row>
-    <row r="5" spans="1:11" ht="99" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
@@ -1656,17 +1645,17 @@
         <v>19</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -1682,18 +1671,18 @@
       <c r="E6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" ht="99" x14ac:dyDescent="0.25">
+      <c r="F6" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="31"/>
+    </row>
+    <row r="7" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
@@ -1710,17 +1699,17 @@
         <v>27</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11" ht="115.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A8" s="31" t="s">
         <v>28</v>
       </c>
@@ -1737,17 +1726,17 @@
         <v>31</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H8" s="31"/>
       <c r="I8" s="31"/>
       <c r="J8" s="31"/>
       <c r="K8" s="31"/>
     </row>
-    <row r="9" spans="1:11" ht="82.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="84" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
@@ -1757,24 +1746,24 @@
       <c r="C9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>36</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
@@ -1791,17 +1780,17 @@
         <v>41</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H10" s="31"/>
       <c r="I10" s="31"/>
       <c r="J10" s="31"/>
       <c r="K10" s="31"/>
     </row>
-    <row r="11" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>42</v>
       </c>
@@ -1815,27 +1804,27 @@
         <v>44</v>
       </c>
       <c r="E11" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>207</v>
-      </c>
       <c r="G11" s="25" t="s">
+        <v>213</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>215</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>217</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" ht="132" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>46</v>
@@ -1844,20 +1833,20 @@
         <v>47</v>
       </c>
       <c r="E12" s="32" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H12" s="31"/>
       <c r="I12" s="31"/>
       <c r="J12" s="31"/>
       <c r="K12" s="31"/>
     </row>
-    <row r="13" spans="1:11" ht="198" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>48</v>
       </c>
@@ -1874,21 +1863,21 @@
         <v>52</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="G13" s="44" t="s">
-        <v>215</v>
+        <v>205</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>213</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="82.5" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="84" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>53</v>
       </c>
@@ -1905,17 +1894,17 @@
         <v>57</v>
       </c>
       <c r="F14" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H14" s="31"/>
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
       <c r="K14" s="31"/>
     </row>
-    <row r="15" spans="1:11" ht="66" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>58</v>
       </c>
@@ -1932,17 +1921,17 @@
         <v>62</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:11" ht="82.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="84" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>63</v>
       </c>
@@ -1959,17 +1948,17 @@
         <v>67</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H16" s="31"/>
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
       <c r="K16" s="31"/>
     </row>
-    <row r="17" spans="1:11" ht="66" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>68</v>
       </c>
@@ -1986,17 +1975,17 @@
         <v>72</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:11" ht="115.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>73</v>
       </c>
@@ -2010,161 +1999,165 @@
         <v>76</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>77</v>
+        <v>222</v>
       </c>
       <c r="F18" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G18" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H18" s="31"/>
       <c r="I18" s="31"/>
       <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
-    </row>
-    <row r="19" spans="1:11" ht="280.5" x14ac:dyDescent="0.25">
+      <c r="K18" s="31" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="285.60000000000002" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>82</v>
-      </c>
       <c r="F19" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="G19" s="44" t="s">
-        <v>215</v>
-      </c>
-      <c r="H19" s="3"/>
+        <v>205</v>
+      </c>
+      <c r="G19" s="25" t="s">
+        <v>213</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>224</v>
+      </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="E20" s="32" t="s">
         <v>86</v>
       </c>
-      <c r="E20" s="32" t="s">
-        <v>87</v>
-      </c>
       <c r="F20" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H20" s="31"/>
       <c r="I20" s="31"/>
       <c r="J20" s="31"/>
       <c r="K20" s="31"/>
     </row>
-    <row r="21" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="F21" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:11" ht="82.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="84" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="E22" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="E22" s="32" t="s">
-        <v>97</v>
-      </c>
       <c r="F22" s="31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H22" s="31"/>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
       <c r="K22" s="31"/>
     </row>
-    <row r="23" spans="1:11" ht="82.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="84" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="E23" s="5" t="s">
-        <v>102</v>
-      </c>
       <c r="F23" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -2177,283 +2170,283 @@
       <c r="J24" s="34"/>
       <c r="K24" s="34"/>
     </row>
-    <row r="25" spans="1:11" ht="115.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="E25" s="10" t="s">
-        <v>108</v>
-      </c>
       <c r="F25" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
     </row>
-    <row r="26" spans="1:11" ht="132" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="C26" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="D26" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="D26" s="12" t="s">
+      <c r="E26" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="E26" s="35" t="s">
-        <v>113</v>
-      </c>
       <c r="F26" s="36" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H26" s="36"/>
       <c r="I26" s="36"/>
       <c r="J26" s="36"/>
       <c r="K26" s="36"/>
     </row>
-    <row r="27" spans="1:11" ht="132" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="D27" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>118</v>
-      </c>
       <c r="F27" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G27" s="25" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="148.5" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B28" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="C28" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="D28" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="E28" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="E28" s="35" t="s">
-        <v>123</v>
-      </c>
       <c r="F28" s="36" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H28" s="36"/>
       <c r="I28" s="36"/>
       <c r="J28" s="36"/>
       <c r="K28" s="36"/>
     </row>
-    <row r="29" spans="1:11" ht="148.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="C29" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="E29" s="10" t="s">
-        <v>127</v>
-      </c>
       <c r="F29" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="1:11" ht="198" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="C30" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="D30" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="E30" s="35" t="s">
         <v>131</v>
       </c>
-      <c r="E30" s="35" t="s">
-        <v>132</v>
-      </c>
       <c r="F30" s="36" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G30" s="36" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H30" s="36"/>
       <c r="I30" s="36"/>
       <c r="J30" s="36"/>
       <c r="K30" s="36"/>
     </row>
-    <row r="31" spans="1:11" ht="181.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B31" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="C31" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="D31" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="E31" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="E31" s="16" t="s">
-        <v>137</v>
-      </c>
       <c r="F31" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
     </row>
-    <row r="32" spans="1:11" ht="99" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="C32" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B32" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="C32" s="13" t="s">
+      <c r="D32" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="E32" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="E32" s="35" t="s">
-        <v>141</v>
-      </c>
       <c r="F32" s="36" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G32" s="36" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H32" s="36"/>
       <c r="I32" s="36"/>
       <c r="J32" s="36"/>
       <c r="K32" s="36"/>
     </row>
-    <row r="33" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C33" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="C33" s="10" t="s">
+      <c r="D33" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="E33" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="E33" s="10" t="s">
-        <v>145</v>
-      </c>
       <c r="F33" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="C34" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="B34" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="C34" s="13" t="s">
+      <c r="D34" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="E34" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="E34" s="35" t="s">
-        <v>149</v>
-      </c>
       <c r="F34" s="36" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G34" s="36" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H34" s="36"/>
       <c r="I34" s="36"/>
       <c r="J34" s="36"/>
       <c r="K34" s="36"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B35" s="18"/>
       <c r="C35" s="18"/>
@@ -2466,283 +2459,283 @@
       <c r="J35" s="38"/>
       <c r="K35" s="38"/>
     </row>
-    <row r="36" spans="1:11" ht="132" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="C36" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="D36" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>154</v>
-      </c>
       <c r="E36" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
     </row>
-    <row r="37" spans="1:11" ht="132" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A37" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="B37" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="B37" s="20" t="s">
+      <c r="C37" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="C37" s="21" t="s">
+      <c r="D37" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="D37" s="20" t="s">
-        <v>158</v>
-      </c>
       <c r="E37" s="39" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F37" s="40" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G37" s="40" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H37" s="40"/>
       <c r="I37" s="40"/>
       <c r="J37" s="40"/>
       <c r="K37" s="40"/>
     </row>
-    <row r="38" spans="1:11" ht="132" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B38" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="C38" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="D38" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="C38" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>161</v>
-      </c>
       <c r="E38" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G38" s="25" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>162</v>
+        <v>225</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
       <c r="K38" s="5" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="148.5" x14ac:dyDescent="0.25">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A39" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="C39" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="B39" s="20" t="s">
+      <c r="D39" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="C39" s="21" t="s">
-        <v>165</v>
-      </c>
-      <c r="D39" s="20" t="s">
-        <v>166</v>
-      </c>
       <c r="E39" s="39" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F39" s="40" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G39" s="40" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H39" s="40"/>
       <c r="I39" s="40"/>
       <c r="J39" s="40"/>
       <c r="K39" s="40"/>
     </row>
-    <row r="40" spans="1:11" ht="148.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D40" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B40" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="C40" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>169</v>
-      </c>
       <c r="E40" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
     </row>
-    <row r="41" spans="1:11" ht="198" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A41" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>169</v>
+      </c>
+      <c r="C41" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="B41" s="20" t="s">
+      <c r="D41" s="20" t="s">
         <v>171</v>
       </c>
-      <c r="C41" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="D41" s="20" t="s">
-        <v>173</v>
-      </c>
       <c r="E41" s="39" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F41" s="40" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G41" s="40" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H41" s="40"/>
       <c r="I41" s="40"/>
       <c r="J41" s="40"/>
       <c r="K41" s="40"/>
     </row>
-    <row r="42" spans="1:11" ht="181.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A42" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="C42" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="B42" s="15" t="s">
+      <c r="D42" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="C42" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="D42" s="15" t="s">
-        <v>177</v>
-      </c>
       <c r="E42" s="16" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
     </row>
-    <row r="43" spans="1:11" ht="99" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A43" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="D43" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="B43" s="20" t="s">
-        <v>202</v>
-      </c>
-      <c r="C43" s="21" t="s">
-        <v>179</v>
-      </c>
-      <c r="D43" s="20" t="s">
-        <v>180</v>
-      </c>
       <c r="E43" s="39" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F43" s="40" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G43" s="40" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H43" s="40"/>
       <c r="I43" s="40"/>
       <c r="J43" s="40"/>
       <c r="K43" s="40"/>
     </row>
-    <row r="44" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="D44" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="B44" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>183</v>
-      </c>
       <c r="E44" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H44" s="3"/>
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
     </row>
-    <row r="45" spans="1:11" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A45" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="D45" s="20" t="s">
         <v>184</v>
       </c>
-      <c r="B45" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="C45" s="21" t="s">
-        <v>185</v>
-      </c>
-      <c r="D45" s="20" t="s">
-        <v>186</v>
-      </c>
       <c r="E45" s="39" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F45" s="40" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G45" s="40" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H45" s="40"/>
       <c r="I45" s="40"/>
       <c r="J45" s="40"/>
       <c r="K45" s="40"/>
     </row>
-    <row r="46" spans="1:11" ht="33" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B46" s="23"/>
       <c r="C46" s="24"/>
@@ -2755,54 +2748,54 @@
       <c r="J46" s="42"/>
       <c r="K46" s="42"/>
     </row>
-    <row r="47" spans="1:11" ht="115.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C47" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="D47" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="E47" s="10" t="s">
         <v>190</v>
       </c>
-      <c r="D47" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="E47" s="10" t="s">
-        <v>192</v>
-      </c>
       <c r="F47" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H47" s="3"/>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
     </row>
-    <row r="48" spans="1:11" ht="132" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C48" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="D48" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="E48" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="D48" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>197</v>
-      </c>
       <c r="F48" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H48" s="3"/>
       <c r="I48" s="3"/>

</xml_diff>

<commit_message>
SCRUM-82: bo sung noi dung codeceptjs
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Test_Case_Report_FE.xlsx
+++ b/Docs/QA-Testing/Test_Case_Report_FE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiemChungPhanMem\Docs\QA-Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C33D1E3-AB95-42CB-A3D1-3C7E9A057C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77FB11DA-1FE0-4329-8AA5-93469161C9D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="229">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -901,9 +901,6 @@
     <t>Assertion $40.00 thất bại vì subtotal hiển thị $40,140.00 (dữ liệu giỏ / format số bị ảnh hưởng bởi data BVA trước đó hoặc locale). Không phải bug nghiệp vụ Add to Cart. Cần reset DB hoặc sửa expected linh hoạt hơn trước khi retest.</t>
   </si>
   <si>
-    <t>Sau Checkout hệ thống chuyển về trang chủ (Get Whatever You Want!). Test vẫn expect thấy "Spring In Action" trên trang sau checkout → sai expected. Hành vi thực tế đúng (cart cleared, redirect home). Sửa test: expect trang chủ hoặc thông báo thành công, không expect tên SP trên /cart nữa.</t>
-  </si>
-  <si>
     <t>Thấy "Cenceled" (typo UI) – liên quan SCRUM-52, không làm fail case này.</t>
   </si>
   <si>
@@ -923,6 +920,18 @@
   </si>
   <si>
     <t>SCRUM-44(đã fix)-SCRUM-81(chưa fix)</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>Codecept</t>
+  </si>
+  <si>
+    <t>Đã sửa assert; hành vi redirect về trang chủ (Home) là chính xác.</t>
+  </si>
+  <si>
+    <t>Chạy tự động thành công.</t>
   </si>
 </sst>
 </file>
@@ -1507,24 +1516,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="16.8" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.6640625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="36" style="6" customWidth="1"/>
-    <col min="3" max="3" width="30.109375" style="6" customWidth="1" outlineLevel="1"/>
-    <col min="4" max="4" width="52.88671875" style="6" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="47.88671875" style="6" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="6" width="12.109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.88671875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6640625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16.109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5546875" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="34.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.21875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48" style="6" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="68.21875" style="6" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="75.21875" style="6" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="16.77734375" style="1" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="7" max="7" width="28.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="33.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
@@ -1550,16 +1560,19 @@
         <v>208</v>
       </c>
       <c r="I1" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="J1" s="27" t="s">
         <v>209</v>
       </c>
-      <c r="J1" s="27" t="s">
+      <c r="K1" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="K1" s="27" t="s">
+      <c r="L1" s="27" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
         <v>5</v>
       </c>
@@ -1573,8 +1586,9 @@
       <c r="I2" s="30"/>
       <c r="J2" s="30"/>
       <c r="K2" s="30"/>
-    </row>
-    <row r="3" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="L2" s="30"/>
+    </row>
+    <row r="3" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -1597,11 +1611,16 @@
         <v>212</v>
       </c>
       <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="L3" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A4" s="31" t="s">
         <v>10</v>
       </c>
@@ -1624,11 +1643,16 @@
         <v>212</v>
       </c>
       <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
+      <c r="I4" s="31" t="s">
+        <v>226</v>
+      </c>
       <c r="J4" s="31"/>
       <c r="K4" s="31"/>
-    </row>
-    <row r="5" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="L4" s="31" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
@@ -1651,11 +1675,14 @@
         <v>212</v>
       </c>
       <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -1681,8 +1708,9 @@
       <c r="I6" s="31"/>
       <c r="J6" s="31"/>
       <c r="K6" s="31"/>
-    </row>
-    <row r="7" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="L6" s="31"/>
+    </row>
+    <row r="7" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>24</v>
       </c>
@@ -1708,8 +1736,9 @@
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
-    </row>
-    <row r="8" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
+      <c r="L7" s="3"/>
+    </row>
+    <row r="8" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A8" s="31" t="s">
         <v>28</v>
       </c>
@@ -1735,8 +1764,9 @@
       <c r="I8" s="31"/>
       <c r="J8" s="31"/>
       <c r="K8" s="31"/>
-    </row>
-    <row r="9" spans="1:11" ht="84" x14ac:dyDescent="0.3">
+      <c r="L8" s="31"/>
+    </row>
+    <row r="9" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
@@ -1759,11 +1789,14 @@
         <v>212</v>
       </c>
       <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
+      <c r="I9" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
@@ -1786,11 +1819,14 @@
         <v>212</v>
       </c>
       <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
+      <c r="I10" s="31" t="s">
+        <v>226</v>
+      </c>
       <c r="J10" s="31"/>
       <c r="K10" s="31"/>
-    </row>
-    <row r="11" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L10" s="31"/>
+    </row>
+    <row r="11" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>42</v>
       </c>
@@ -1818,8 +1854,9 @@
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>45</v>
       </c>
@@ -1845,8 +1882,9 @@
       <c r="I12" s="31"/>
       <c r="J12" s="31"/>
       <c r="K12" s="31"/>
-    </row>
-    <row r="13" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="L12" s="31"/>
+    </row>
+    <row r="13" spans="1:12" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>48</v>
       </c>
@@ -1869,15 +1907,18 @@
         <v>213</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="I13" s="3"/>
+        <v>222</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J13" s="3"/>
-      <c r="K13" s="3" t="s">
+      <c r="K13" s="3"/>
+      <c r="L13" s="3" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="84" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>53</v>
       </c>
@@ -1903,8 +1944,9 @@
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
       <c r="K14" s="31"/>
-    </row>
-    <row r="15" spans="1:11" ht="67.2" x14ac:dyDescent="0.3">
+      <c r="L14" s="31"/>
+    </row>
+    <row r="15" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>58</v>
       </c>
@@ -1927,11 +1969,14 @@
         <v>212</v>
       </c>
       <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
+      <c r="I15" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" ht="84" x14ac:dyDescent="0.3">
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>63</v>
       </c>
@@ -1957,8 +2002,9 @@
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
       <c r="K16" s="31"/>
-    </row>
-    <row r="17" spans="1:11" ht="67.2" x14ac:dyDescent="0.3">
+      <c r="L16" s="31"/>
+    </row>
+    <row r="17" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>68</v>
       </c>
@@ -1981,11 +2027,14 @@
         <v>212</v>
       </c>
       <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
+      <c r="I17" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
-    </row>
-    <row r="18" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>73</v>
       </c>
@@ -1999,7 +2048,7 @@
         <v>76</v>
       </c>
       <c r="E18" s="32" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F18" s="31" t="s">
         <v>205</v>
@@ -2010,11 +2059,12 @@
       <c r="H18" s="31"/>
       <c r="I18" s="31"/>
       <c r="J18" s="31"/>
-      <c r="K18" s="31" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="285.60000000000002" x14ac:dyDescent="0.3">
+      <c r="K18" s="31"/>
+      <c r="L18" s="31" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>77</v>
       </c>
@@ -2037,15 +2087,18 @@
         <v>213</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="I19" s="3"/>
+        <v>223</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J19" s="3"/>
-      <c r="K19" s="3" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="K19" s="3"/>
+      <c r="L19" s="3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>82</v>
       </c>
@@ -2068,11 +2121,14 @@
         <v>212</v>
       </c>
       <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
+      <c r="I20" s="31" t="s">
+        <v>226</v>
+      </c>
       <c r="J20" s="31"/>
       <c r="K20" s="31"/>
-    </row>
-    <row r="21" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L20" s="31"/>
+    </row>
+    <row r="21" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>87</v>
       </c>
@@ -2098,8 +2154,9 @@
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
-    </row>
-    <row r="22" spans="1:11" ht="84" x14ac:dyDescent="0.3">
+      <c r="L21" s="3"/>
+    </row>
+    <row r="22" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>92</v>
       </c>
@@ -2125,8 +2182,9 @@
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
       <c r="K22" s="31"/>
-    </row>
-    <row r="23" spans="1:11" ht="84" x14ac:dyDescent="0.3">
+      <c r="L22" s="31"/>
+    </row>
+    <row r="23" spans="1:12" ht="67.2" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>97</v>
       </c>
@@ -2149,13 +2207,16 @@
         <v>212</v>
       </c>
       <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
+      <c r="I23" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J23" s="3"/>
-      <c r="K23" s="3" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K23" s="3"/>
+      <c r="L23" s="3" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>102</v>
       </c>
@@ -2169,8 +2230,9 @@
       <c r="I24" s="34"/>
       <c r="J24" s="34"/>
       <c r="K24" s="34"/>
-    </row>
-    <row r="25" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
+      <c r="L24" s="34"/>
+    </row>
+    <row r="25" spans="1:12" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>103</v>
       </c>
@@ -2196,8 +2258,9 @@
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
-    </row>
-    <row r="26" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
+      <c r="L25" s="3"/>
+    </row>
+    <row r="26" spans="1:12" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>108</v>
       </c>
@@ -2223,8 +2286,9 @@
       <c r="I26" s="36"/>
       <c r="J26" s="36"/>
       <c r="K26" s="36"/>
-    </row>
-    <row r="27" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
+      <c r="L26" s="36"/>
+    </row>
+    <row r="27" spans="1:12" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>113</v>
       </c>
@@ -2247,15 +2311,16 @@
         <v>213</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
-      <c r="K27" s="3" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
+      <c r="K27" s="3"/>
+      <c r="L27" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>118</v>
       </c>
@@ -2281,8 +2346,9 @@
       <c r="I28" s="36"/>
       <c r="J28" s="36"/>
       <c r="K28" s="36"/>
-    </row>
-    <row r="29" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
+      <c r="L28" s="36"/>
+    </row>
+    <row r="29" spans="1:12" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>123</v>
       </c>
@@ -2308,8 +2374,9 @@
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
-    </row>
-    <row r="30" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="L29" s="3"/>
+    </row>
+    <row r="30" spans="1:12" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
         <v>127</v>
       </c>
@@ -2332,11 +2399,14 @@
         <v>212</v>
       </c>
       <c r="H30" s="36"/>
-      <c r="I30" s="36"/>
+      <c r="I30" s="36" t="s">
+        <v>226</v>
+      </c>
       <c r="J30" s="36"/>
       <c r="K30" s="36"/>
-    </row>
-    <row r="31" spans="1:11" ht="184.8" x14ac:dyDescent="0.3">
+      <c r="L30" s="36"/>
+    </row>
+    <row r="31" spans="1:12" ht="168" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>132</v>
       </c>
@@ -2362,8 +2432,9 @@
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
-    </row>
-    <row r="32" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="L31" s="3"/>
+    </row>
+    <row r="32" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
         <v>137</v>
       </c>
@@ -2389,8 +2460,9 @@
       <c r="I32" s="36"/>
       <c r="J32" s="36"/>
       <c r="K32" s="36"/>
-    </row>
-    <row r="33" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L32" s="36"/>
+    </row>
+    <row r="33" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>141</v>
       </c>
@@ -2416,8 +2488,9 @@
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
-    </row>
-    <row r="34" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L33" s="3"/>
+    </row>
+    <row r="34" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
         <v>145</v>
       </c>
@@ -2443,8 +2516,9 @@
       <c r="I34" s="36"/>
       <c r="J34" s="36"/>
       <c r="K34" s="36"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L34" s="36"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="17" t="s">
         <v>149</v>
       </c>
@@ -2458,8 +2532,9 @@
       <c r="I35" s="38"/>
       <c r="J35" s="38"/>
       <c r="K35" s="38"/>
-    </row>
-    <row r="36" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
+      <c r="L35" s="38"/>
+    </row>
+    <row r="36" spans="1:12" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>150</v>
       </c>
@@ -2485,8 +2560,9 @@
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
-    </row>
-    <row r="37" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
+      <c r="L36" s="3"/>
+    </row>
+    <row r="37" spans="1:12" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A37" s="19" t="s">
         <v>154</v>
       </c>
@@ -2512,8 +2588,9 @@
       <c r="I37" s="40"/>
       <c r="J37" s="40"/>
       <c r="K37" s="40"/>
-    </row>
-    <row r="38" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
+      <c r="L37" s="40"/>
+    </row>
+    <row r="38" spans="1:12" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>158</v>
       </c>
@@ -2536,15 +2613,18 @@
         <v>213</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="I38" s="3"/>
+        <v>224</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J38" s="3"/>
-      <c r="K38" s="5" t="s">
+      <c r="K38" s="3"/>
+      <c r="L38" s="5" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A39" s="19" t="s">
         <v>161</v>
       </c>
@@ -2570,8 +2650,9 @@
       <c r="I39" s="40"/>
       <c r="J39" s="40"/>
       <c r="K39" s="40"/>
-    </row>
-    <row r="40" spans="1:11" ht="151.19999999999999" x14ac:dyDescent="0.3">
+      <c r="L39" s="40"/>
+    </row>
+    <row r="40" spans="1:12" ht="151.19999999999999" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>165</v>
       </c>
@@ -2597,8 +2678,9 @@
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
-    </row>
-    <row r="41" spans="1:11" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="L40" s="3"/>
+    </row>
+    <row r="41" spans="1:12" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A41" s="19" t="s">
         <v>168</v>
       </c>
@@ -2624,8 +2706,9 @@
       <c r="I41" s="40"/>
       <c r="J41" s="40"/>
       <c r="K41" s="40"/>
-    </row>
-    <row r="42" spans="1:11" ht="184.8" x14ac:dyDescent="0.3">
+      <c r="L41" s="40"/>
+    </row>
+    <row r="42" spans="1:12" ht="184.8" x14ac:dyDescent="0.3">
       <c r="A42" s="14" t="s">
         <v>172</v>
       </c>
@@ -2651,8 +2734,9 @@
       <c r="I42" s="3"/>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
-    </row>
-    <row r="43" spans="1:11" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="L42" s="3"/>
+    </row>
+    <row r="43" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A43" s="19" t="s">
         <v>176</v>
       </c>
@@ -2678,8 +2762,9 @@
       <c r="I43" s="40"/>
       <c r="J43" s="40"/>
       <c r="K43" s="40"/>
-    </row>
-    <row r="44" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L43" s="40"/>
+    </row>
+    <row r="44" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>179</v>
       </c>
@@ -2705,8 +2790,9 @@
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
-    </row>
-    <row r="45" spans="1:11" ht="50.4" x14ac:dyDescent="0.3">
+      <c r="L44" s="3"/>
+    </row>
+    <row r="45" spans="1:12" ht="50.4" x14ac:dyDescent="0.3">
       <c r="A45" s="19" t="s">
         <v>182</v>
       </c>
@@ -2732,8 +2818,9 @@
       <c r="I45" s="40"/>
       <c r="J45" s="40"/>
       <c r="K45" s="40"/>
-    </row>
-    <row r="46" spans="1:11" ht="33.6" x14ac:dyDescent="0.3">
+      <c r="L45" s="40"/>
+    </row>
+    <row r="46" spans="1:12" ht="33.6" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
         <v>185</v>
       </c>
@@ -2747,8 +2834,9 @@
       <c r="I46" s="42"/>
       <c r="J46" s="42"/>
       <c r="K46" s="42"/>
-    </row>
-    <row r="47" spans="1:11" ht="117.6" x14ac:dyDescent="0.3">
+      <c r="L46" s="42"/>
+    </row>
+    <row r="47" spans="1:12" ht="117.6" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>186</v>
       </c>
@@ -2771,11 +2859,14 @@
         <v>212</v>
       </c>
       <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
+      <c r="I47" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
-    </row>
-    <row r="48" spans="1:11" ht="134.4" x14ac:dyDescent="0.3">
+      <c r="L47" s="3"/>
+    </row>
+    <row r="48" spans="1:12" ht="84" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>191</v>
       </c>
@@ -2798,9 +2889,12 @@
         <v>212</v>
       </c>
       <c r="H48" s="3"/>
-      <c r="I48" s="3"/>
+      <c r="I48" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>